<commit_message>
dataset cards no formato do modelo da aula
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entregaveis/dataset_card_questoes.xlsx
+++ b/entregaveis/dataset_card_questoes.xlsx
@@ -93,7 +93,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -106,6 +106,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -515,11 +518,12 @@
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Dataset Card - QuestõesTI-FGV</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Questões de Concursos de TI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1"/>
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Atributo</t>
@@ -530,13 +534,9 @@
           <t>Descrição</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1">
+      <c r="C3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">   Nome do Dataset:</t>
@@ -549,7 +549,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>QuestõesTI-FGV</t>
+          <t>Corpus de Questões de Concursos de TI (QuestõesTI-FGV)</t>
         </is>
       </c>
     </row>
@@ -581,13 +581,13 @@
           <t>Atributo contendo informações sobre onde pode ser obtido e como. Pode ser simplesmente a URL de onde está hospedado: git, hugging face, ...</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://github.com/barbaradasilvadapper/T1-PLN </t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/barbaradasilvadapper/T1-PLN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">   Versão e Data de criação</t>
@@ -604,7 +604,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">   Versão e Data de atualização</t>
@@ -617,11 +617,11 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>Versão 1.1 - atualizada em 02/10/2026 (classificação de subárea em duas etapas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="135" customHeight="1">
+          <t>Versão 1.1 - atualizada em 02/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Natureza dos documentos:</t>
@@ -634,11 +634,11 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>O dataset foi construído a partir de provas de concursos públicos disponibilizadas na web. A fonte foi o PCI Concursos (https://www.pciconcursos.com.br/provas/ti/). A coleta foi realizada em setembro de 2026: foram selecionadas 95 provas de cargos de TI da banca FGV, com os respectivos gabaritos, baixadas manualmente. Os concursos das provas referem-se aos anos de 2021 a 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
+          <t>Questões de múltipla escolha de 95 provas de TI da banca FGV (2021 a 2026), baixadas do PCI Concursos com os gabaritos e convertidas de PDF para texto. Cada questão tem enunciado, alternativas, gabarito, ano e subárea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
           <t>Domínio:</t>
@@ -651,11 +651,11 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Computação / Tecnologia da Informação (questões de concursos públicos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
+          <t>Computação / Tecnologia da Informação</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Tarefa:</t>
@@ -668,11 +668,11 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>Classificação de Texto (subárea da questão); também serve para resposta a questões de múltipla escolha</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
+          <t>Classificação de Texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Idioma:</t>
@@ -685,11 +685,11 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>Português (Brasil), com termos técnicos em inglês</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="75" customHeight="1">
+          <t>Português (Brasil)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Formato:</t>
@@ -702,7 +702,7 @@
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>JSON, o dataset está organizado em questões (corpus.json: metadados + lista de questões com enunciado, alternativas, gabarito, subárea e ano; por_subarea/*.json: questões agrupadas por ano). Também em CSV e um TXT por questão.</t>
+          <t>JSON (também em CSV)</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" ht="105" customHeight="1">
+    <row r="18" ht="90" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Distribuição em classes:</t>
@@ -779,7 +779,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>O dataset possui questões de 5 subáreas da computação: Eng. Software e Programação: 727 questões (29,0%); Redes e Infraestrutura: 669 questões (26,7%); Segurança da Informação: 502 questões (20,0%); Banco de Dados e Ciência de Dados: 469 questões (18,7%); Governança e Gestão de TI: 139 questões (5,5%). As três primeiras atendem ao mínimo de 500 questões; as duas últimas são subáreas extras.</t>
+          <t>O dataset possui questões de 5 subáreas: Engenharia de Software e Programação (727, 29,0%), Redes e Infraestrutura (669, 26,7%), Segurança da Informação (502, 20,0%), Banco de Dados e Ciência de Dados (469, 18,7%) e Governança e Gestão de TI (139, 5,5%).</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>Tamanho médio em tokens de cada questão (enunciado + alternativas): 106,71</t>
+          <t>Tamanho médio em tokens de cada questão: 106,71 (enunciado + alternativas)</t>
         </is>
       </c>
     </row>
@@ -841,8 +841,10 @@
           <t>Dado numérico que indica, por exemplo, a quantidade de palavras corretas identificadas no dataset</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n">
-        <v>0.947</v>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>94,7% das palavras reconhecidas em dicionário (português e inglês)</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
@@ -858,11 +860,11 @@
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>5.2 MB (corpus.json)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="409.5" customHeight="1">
+          <t>5,2 MB</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
           <t>Outras informações:</t>
@@ -875,14 +877,11 @@
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>A qualidade dos textos é a proporção de tokens alfabéticos reconhecidos em dicionário de português ou inglês (pyspellchecker); é um limite inferior, pois siglas e termos técnicos (ex.: tcp, json, kubernetes) contam como não reconhecidos. A subárea é atribuída em duas etapas (scripts/subareas.py): pontuação por palavras-chave, com o enunciado valendo o dobro das alternativas; nas questões ambíguas (margem &lt; 4 pontos entre as duas primeiras subáreas), um TF-IDF + k-NN (k=3) treinado nas questões não ambíguas decide. Numa amostra aleatória de 100 questões conferida à mão, 97 estão na subárea correta (dados/validacao_rotulos.csv).</t>
+          <t>Tokens contados via regex de sequências de letras e números. Subárea definida por palavras-chave e k-NN; 97 de 100 questões conferidas estavam corretas.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
 </worksheet>
 </file>
</xml_diff>